<commit_message>
Update locus Quality control and fix herd year assignment
</commit_message>
<xml_diff>
--- a/tables/GD_Tables.xlsx
+++ b/tables/GD_Tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\R_WD\woodbison\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99293F90-AF89-4F2E-8274-FAF5936B4200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A32AEB4-69D2-4BE5-8286-0D8594AD795F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-118" yWindow="-118" windowWidth="20343" windowHeight="12934" xr2:uid="{B9F98977-E913-45D8-AD8A-7C651BE01622}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="148">
   <si>
     <t>Population</t>
   </si>
@@ -530,6 +530,12 @@
       </rPr>
       <t>IS</t>
     </r>
+  </si>
+  <si>
+    <t>0.54 ± 0.20</t>
+  </si>
+  <si>
+    <t>0.53 ± 0.20</t>
   </si>
 </sst>
 </file>
@@ -684,7 +690,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -734,23 +740,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -758,30 +749,50 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1128,37 +1139,37 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:18" ht="17.05" x14ac:dyDescent="0.35">
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="32" t="s">
         <v>137</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21" t="s">
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35" t="s">
         <v>142</v>
       </c>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21" t="s">
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35" t="s">
         <v>143</v>
       </c>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21" t="s">
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22" t="s">
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+      <c r="P2" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
+      <c r="Q2" s="36"/>
+      <c r="R2" s="36"/>
     </row>
     <row r="3" spans="3:18" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C3" s="23"/>
+      <c r="C3" s="32"/>
       <c r="D3" s="18" t="s">
         <v>2</v>
       </c>
@@ -1806,72 +1817,72 @@
       </c>
     </row>
     <row r="19" spans="3:17" ht="17.7" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="29" t="s">
+      <c r="D19" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="E19" s="30" t="s">
+      <c r="E19" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="F19" s="30" t="s">
+      <c r="F19" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="G19" s="30" t="s">
+      <c r="G19" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="H19" s="30" t="s">
+      <c r="H19" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="I19" s="30" t="s">
+      <c r="I19" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="K19" s="31" t="s">
+      <c r="K19" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="L19" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="M19" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="N19" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="O19" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="P19" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q19" s="27" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="C20" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20" s="17">
+        <v>63</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="H20" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="I20" s="17">
         <v>0</v>
       </c>
-      <c r="L19" s="32" t="s">
-        <v>138</v>
-      </c>
-      <c r="M19" s="33" t="s">
-        <v>1</v>
-      </c>
-      <c r="N19" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="O19" s="33" t="s">
-        <v>143</v>
-      </c>
-      <c r="P19" s="33" t="s">
-        <v>144</v>
-      </c>
-      <c r="Q19" s="33" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="20" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C20" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="E20" s="25">
-        <v>63</v>
-      </c>
-      <c r="F20" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="G20" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="H20" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="I20" s="25">
-        <v>0</v>
-      </c>
-      <c r="K20" s="36" t="s">
+      <c r="K20" s="28" t="s">
         <v>5</v>
       </c>
       <c r="L20" s="17" t="s">
@@ -1889,33 +1900,33 @@
       <c r="P20" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="Q20" s="17">
+      <c r="Q20" s="38">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C21" s="26" t="s">
+      <c r="C21" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D21" s="27" t="s">
+      <c r="D21" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="E21" s="27">
+      <c r="E21" s="16">
         <v>20</v>
       </c>
-      <c r="F21" s="27" t="s">
+      <c r="F21" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="G21" s="27" t="s">
+      <c r="G21" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="27" t="s">
+      <c r="H21" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="I21" s="27">
+      <c r="I21" s="16">
         <v>-0.05</v>
       </c>
-      <c r="K21" s="36" t="s">
+      <c r="K21" s="28" t="s">
         <v>18</v>
       </c>
       <c r="L21" s="16" t="s">
@@ -1933,33 +1944,33 @@
       <c r="P21" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="Q21" s="16">
+      <c r="Q21" s="39">
         <v>-0.05</v>
       </c>
     </row>
     <row r="22" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E22" s="25">
+      <c r="E22" s="17">
         <v>39</v>
       </c>
-      <c r="F22" s="25" t="s">
+      <c r="F22" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="G22" s="25" t="s">
+      <c r="G22" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="25" t="s">
+      <c r="H22" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="I22" s="25">
+      <c r="I22" s="17">
         <v>0.02</v>
       </c>
-      <c r="K22" s="37" t="s">
+      <c r="K22" s="29" t="s">
         <v>19</v>
       </c>
       <c r="L22" s="17" t="s">
@@ -1977,31 +1988,31 @@
       <c r="P22" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="Q22" s="17">
+      <c r="Q22" s="38">
         <v>0.02</v>
       </c>
     </row>
     <row r="23" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C23" s="34"/>
-      <c r="D23" s="25" t="s">
+      <c r="C23" s="33"/>
+      <c r="D23" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="17">
         <v>40</v>
       </c>
-      <c r="F23" s="25" t="s">
+      <c r="F23" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="G23" s="25" t="s">
+      <c r="G23" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="H23" s="25" t="s">
+      <c r="H23" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="I23" s="25">
+      <c r="I23" s="17">
         <v>0</v>
       </c>
-      <c r="K23" s="37"/>
+      <c r="K23" s="29"/>
       <c r="L23" s="16" t="s">
         <v>3</v>
       </c>
@@ -2017,31 +2028,31 @@
       <c r="P23" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="Q23" s="16">
+      <c r="Q23" s="39">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C24" s="34"/>
-      <c r="D24" s="25" t="s">
+      <c r="C24" s="33"/>
+      <c r="D24" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="25">
+      <c r="E24" s="17">
         <v>19</v>
       </c>
-      <c r="F24" s="25" t="s">
+      <c r="F24" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="G24" s="25" t="s">
+      <c r="G24" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="25" t="s">
+      <c r="H24" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="I24" s="25">
+      <c r="I24" s="17">
         <v>-0.01</v>
       </c>
-      <c r="K24" s="37"/>
+      <c r="K24" s="29"/>
       <c r="L24" s="17" t="s">
         <v>4</v>
       </c>
@@ -2057,33 +2068,33 @@
       <c r="P24" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="Q24" s="17">
+      <c r="Q24" s="38">
         <v>-0.01</v>
       </c>
     </row>
     <row r="25" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C25" s="26" t="s">
+      <c r="C25" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D25" s="27" t="s">
+      <c r="D25" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="27">
+      <c r="E25" s="16">
         <v>31</v>
       </c>
-      <c r="F25" s="27" t="s">
+      <c r="F25" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="G25" s="27" t="s">
+      <c r="G25" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="H25" s="27" t="s">
+      <c r="H25" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="I25" s="27">
+      <c r="I25" s="16">
         <v>-0.01</v>
       </c>
-      <c r="K25" s="36" t="s">
+      <c r="K25" s="28" t="s">
         <v>20</v>
       </c>
       <c r="L25" s="16" t="s">
@@ -2101,33 +2112,33 @@
       <c r="P25" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="Q25" s="16">
+      <c r="Q25" s="39">
         <v>-0.01</v>
       </c>
     </row>
     <row r="26" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="D26" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="17">
         <v>33</v>
       </c>
-      <c r="F26" s="25" t="s">
+      <c r="F26" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="G26" s="25" t="s">
+      <c r="G26" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="H26" s="25" t="s">
+      <c r="H26" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="I26" s="25">
+      <c r="I26" s="17">
         <v>0</v>
       </c>
-      <c r="K26" s="37" t="s">
+      <c r="K26" s="29" t="s">
         <v>21</v>
       </c>
       <c r="L26" s="17" t="s">
@@ -2145,31 +2156,31 @@
       <c r="P26" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="Q26" s="17">
+      <c r="Q26" s="38">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C27" s="34"/>
-      <c r="D27" s="25" t="s">
+      <c r="C27" s="33"/>
+      <c r="D27" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="25">
+      <c r="E27" s="17">
         <v>20</v>
       </c>
-      <c r="F27" s="25" t="s">
+      <c r="F27" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="G27" s="25" t="s">
+      <c r="G27" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="H27" s="25" t="s">
+      <c r="H27" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="I27" s="25">
+      <c r="I27" s="17">
         <v>0.02</v>
       </c>
-      <c r="K27" s="37"/>
+      <c r="K27" s="29"/>
       <c r="L27" s="16" t="s">
         <v>4</v>
       </c>
@@ -2185,33 +2196,33 @@
       <c r="P27" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="Q27" s="16">
+      <c r="Q27" s="39">
         <v>0.02</v>
       </c>
     </row>
     <row r="28" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C28" s="35" t="s">
+      <c r="C28" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="D28" s="27" t="s">
+      <c r="D28" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E28" s="27">
+      <c r="E28" s="16">
         <v>28</v>
       </c>
-      <c r="F28" s="27" t="s">
+      <c r="F28" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="G28" s="27" t="s">
+      <c r="G28" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="H28" s="27" t="s">
+      <c r="H28" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="I28" s="27">
+      <c r="I28" s="16">
         <v>-0.02</v>
       </c>
-      <c r="K28" s="37" t="s">
+      <c r="K28" s="29" t="s">
         <v>22</v>
       </c>
       <c r="L28" s="17" t="s">
@@ -2229,31 +2240,31 @@
       <c r="P28" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="Q28" s="17">
+      <c r="Q28" s="38">
         <v>-0.02</v>
       </c>
     </row>
     <row r="29" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C29" s="35"/>
-      <c r="D29" s="27" t="s">
+      <c r="C29" s="34"/>
+      <c r="D29" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E29" s="27">
+      <c r="E29" s="16">
         <v>51</v>
       </c>
-      <c r="F29" s="27" t="s">
+      <c r="F29" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="G29" s="27" t="s">
+      <c r="G29" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="H29" s="27" t="s">
+      <c r="H29" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="I29" s="27">
+      <c r="I29" s="16">
         <v>0.01</v>
       </c>
-      <c r="K29" s="37"/>
+      <c r="K29" s="29"/>
       <c r="L29" s="16" t="s">
         <v>3</v>
       </c>
@@ -2269,33 +2280,33 @@
       <c r="P29" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="Q29" s="16">
+      <c r="Q29" s="39">
         <v>0.01</v>
       </c>
     </row>
     <row r="30" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C30" s="24" t="s">
+      <c r="C30" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="D30" s="25" t="s">
+      <c r="D30" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="25">
+      <c r="E30" s="17">
         <v>8</v>
       </c>
-      <c r="F30" s="25" t="s">
+      <c r="F30" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="G30" s="25" t="s">
+      <c r="G30" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="H30" s="25" t="s">
+      <c r="H30" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="I30" s="25">
+      <c r="I30" s="17">
         <v>0.05</v>
       </c>
-      <c r="K30" s="36" t="s">
+      <c r="K30" s="28" t="s">
         <v>23</v>
       </c>
       <c r="L30" s="17" t="s">
@@ -2313,33 +2324,33 @@
       <c r="P30" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="Q30" s="17">
+      <c r="Q30" s="38">
         <v>0.05</v>
       </c>
     </row>
     <row r="31" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C31" s="24" t="s">
+      <c r="C31" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="D31" s="25" t="s">
+      <c r="D31" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="25">
+      <c r="E31" s="17">
         <v>17</v>
       </c>
-      <c r="F31" s="25" t="s">
+      <c r="F31" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="G31" s="25" t="s">
+      <c r="G31" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="H31" s="25" t="s">
+      <c r="H31" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="I31" s="25">
+      <c r="I31" s="17">
         <v>0</v>
       </c>
-      <c r="K31" s="36" t="s">
+      <c r="K31" s="28" t="s">
         <v>24</v>
       </c>
       <c r="L31" s="16" t="s">
@@ -2349,7 +2360,7 @@
         <v>17</v>
       </c>
       <c r="N31" s="16" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="O31" s="16" t="s">
         <v>112</v>
@@ -2357,33 +2368,33 @@
       <c r="P31" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="Q31" s="16">
+      <c r="Q31" s="39">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C32" s="26" t="s">
+      <c r="C32" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="27" t="s">
+      <c r="D32" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E32" s="27">
+      <c r="E32" s="16">
         <v>19</v>
       </c>
-      <c r="F32" s="27" t="s">
+      <c r="F32" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G32" s="27" t="s">
+      <c r="G32" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="H32" s="27" t="s">
+      <c r="H32" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="I32" s="27">
+      <c r="I32" s="16">
         <v>0.01</v>
       </c>
-      <c r="K32" s="37" t="s">
+      <c r="K32" s="29" t="s">
         <v>25</v>
       </c>
       <c r="L32" s="17" t="s">
@@ -2401,33 +2412,33 @@
       <c r="P32" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="Q32" s="17">
+      <c r="Q32" s="38">
         <v>0.01</v>
       </c>
     </row>
     <row r="33" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C33" s="26" t="s">
+      <c r="C33" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D33" s="27" t="s">
+      <c r="D33" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="E33" s="27">
-        <v>29</v>
-      </c>
-      <c r="F33" s="27" t="s">
+      <c r="E33" s="16">
+        <v>29</v>
+      </c>
+      <c r="F33" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="G33" s="27" t="s">
+      <c r="G33" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="H33" s="27" t="s">
+      <c r="H33" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="I33" s="27">
+      <c r="I33" s="16">
         <v>-0.03</v>
       </c>
-      <c r="K33" s="37"/>
+      <c r="K33" s="29"/>
       <c r="L33" s="16" t="s">
         <v>4</v>
       </c>
@@ -2443,33 +2454,33 @@
       <c r="P33" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="Q33" s="16">
+      <c r="Q33" s="39">
         <v>-0.03</v>
       </c>
     </row>
     <row r="34" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C34" s="24" t="s">
+      <c r="C34" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="25" t="s">
+      <c r="D34" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E34" s="25">
+      <c r="E34" s="17">
         <v>10</v>
       </c>
-      <c r="F34" s="25" t="s">
+      <c r="F34" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="G34" s="25" t="s">
+      <c r="G34" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="H34" s="25" t="s">
+      <c r="H34" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="I34" s="25">
+      <c r="I34" s="17">
         <v>0.02</v>
       </c>
-      <c r="K34" s="37" t="s">
+      <c r="K34" s="29" t="s">
         <v>26</v>
       </c>
       <c r="L34" s="17" t="s">
@@ -2487,33 +2498,33 @@
       <c r="P34" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="Q34" s="17">
+      <c r="Q34" s="38">
         <v>0.02</v>
       </c>
     </row>
     <row r="35" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C35" s="24" t="s">
+      <c r="C35" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D35" s="25" t="s">
+      <c r="D35" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E35" s="25">
+      <c r="E35" s="17">
         <v>8</v>
       </c>
-      <c r="F35" s="25" t="s">
+      <c r="F35" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="G35" s="25" t="s">
+      <c r="G35" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="H35" s="25" t="s">
+      <c r="H35" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="I35" s="25">
+      <c r="I35" s="17">
         <v>-0.05</v>
       </c>
-      <c r="K35" s="37"/>
+      <c r="K35" s="29"/>
       <c r="L35" s="16" t="s">
         <v>4</v>
       </c>
@@ -2521,7 +2532,7 @@
         <v>8</v>
       </c>
       <c r="N35" s="16" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="O35" s="16" t="s">
         <v>121</v>
@@ -2529,33 +2540,33 @@
       <c r="P35" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="Q35" s="16">
+      <c r="Q35" s="39">
         <v>-0.05</v>
       </c>
     </row>
     <row r="36" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="27" t="s">
+      <c r="D36" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E36" s="27">
+      <c r="E36" s="16">
         <v>81</v>
       </c>
-      <c r="F36" s="27" t="s">
+      <c r="F36" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="G36" s="27" t="s">
+      <c r="G36" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="H36" s="27" t="s">
+      <c r="H36" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="I36" s="27">
+      <c r="I36" s="16">
         <v>0.02</v>
       </c>
-      <c r="K36" s="37" t="s">
+      <c r="K36" s="29" t="s">
         <v>27</v>
       </c>
       <c r="L36" s="17" t="s">
@@ -2573,7 +2584,7 @@
       <c r="P36" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="Q36" s="17">
+      <c r="Q36" s="38">
         <v>0.02</v>
       </c>
     </row>
@@ -2599,7 +2610,7 @@
       <c r="I37" s="20">
         <v>0.01</v>
       </c>
-      <c r="K37" s="38"/>
+      <c r="K37" s="30"/>
       <c r="L37" s="20" t="s">
         <v>4</v>
       </c>
@@ -2615,33 +2626,33 @@
       <c r="P37" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="Q37" s="20">
+      <c r="Q37" s="40">
         <v>0.01</v>
       </c>
     </row>
     <row r="38" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C38" s="24" t="s">
+      <c r="C38" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="25" t="s">
+      <c r="D38" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="17">
         <v>30</v>
       </c>
-      <c r="F38" s="25" t="s">
+      <c r="F38" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="G38" s="25" t="s">
+      <c r="G38" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="H38" s="25" t="s">
+      <c r="H38" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="I38" s="25">
+      <c r="I38" s="17">
         <v>0.03</v>
       </c>
-      <c r="K38" s="39" t="s">
+      <c r="K38" s="31" t="s">
         <v>28</v>
       </c>
       <c r="L38" s="17" t="s">
@@ -2659,33 +2670,33 @@
       <c r="P38" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="Q38" s="17">
+      <c r="Q38" s="38">
         <v>0.03</v>
       </c>
     </row>
     <row r="39" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C39" s="24" t="s">
+      <c r="C39" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="25" t="s">
+      <c r="D39" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="17">
         <v>32</v>
       </c>
-      <c r="F39" s="25" t="s">
+      <c r="F39" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="G39" s="25" t="s">
+      <c r="G39" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="H39" s="25" t="s">
+      <c r="H39" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="I39" s="25">
+      <c r="I39" s="17">
         <v>0</v>
       </c>
-      <c r="K39" s="37"/>
+      <c r="K39" s="29"/>
       <c r="L39" s="16" t="s">
         <v>3</v>
       </c>
@@ -2701,33 +2712,33 @@
       <c r="P39" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="Q39" s="16">
+      <c r="Q39" s="39">
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="3:17" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="C40" s="24" t="s">
+      <c r="C40" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D40" s="25" t="s">
+      <c r="D40" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E40" s="25">
+      <c r="E40" s="17">
         <v>35</v>
       </c>
-      <c r="F40" s="25" t="s">
+      <c r="F40" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="G40" s="25" t="s">
+      <c r="G40" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="H40" s="25" t="s">
+      <c r="H40" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="I40" s="25">
+      <c r="I40" s="17">
         <v>0.01</v>
       </c>
-      <c r="K40" s="37"/>
+      <c r="K40" s="29"/>
       <c r="L40" s="17" t="s">
         <v>4</v>
       </c>
@@ -2743,12 +2754,15 @@
       <c r="P40" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="Q40" s="17">
+      <c r="Q40" s="38">
         <v>0.01</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="P2:R2"/>
     <mergeCell ref="K32:K33"/>
     <mergeCell ref="K34:K35"/>
     <mergeCell ref="K36:K37"/>
@@ -2762,9 +2776,6 @@
     <mergeCell ref="K28:K29"/>
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="P2:R2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>